<commit_message>
docs: explain Study 002 quality proxy workflow source
</commit_message>
<xml_diff>
--- a/research/study_002_foundation_model_comparison/analysis/statistical_outputs/measurement_validity_audit.xlsx
+++ b/research/study_002_foundation_model_comparison/analysis/statistical_outputs/measurement_validity_audit.xlsx
@@ -434,7 +434,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B11"/>
+  <dimension ref="A1:B13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="41" customWidth="1" min="1" max="1"/>
@@ -550,10 +550,34 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
+          <t>Workflow design note</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Basic Agent and Planner-Executor have no reviewer stage; their V1.4.4 parsing logic uses confidence as the quality_score fallback when no parsed quality_score is emitted.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Reviewer workflow note</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Planner-Executor-Reviewer includes a reviewer stage that emits a review-derived quality_score, allowing quality_score and confidence to diverge.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
           <t>Interpretation note</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="B13" t="inlineStr">
         <is>
           <t>High equality rates indicate confidence-aligned operational scoring rather than independent human quality judgment.</t>
         </is>

</xml_diff>